<commit_message>
fix: correct plate validation and filter invalid plates from reports
</commit_message>
<xml_diff>
--- a/reports/plate_report.xlsx
+++ b/reports/plate_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,6 +446,50 @@
         <is>
           <t>Seconds</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ABC128</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ABC288</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>